<commit_message>
new results and analysis / aggregation charts
</commit_message>
<xml_diff>
--- a/0_Threshold_OUTPUT/direct_A0A072Z841_Corynebacterium_glutamicum_ATCC_13032.xlsx
+++ b/0_Threshold_OUTPUT/direct_A0A072Z841_Corynebacterium_glutamicum_ATCC_13032.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,6 +469,11 @@
           <t>p_value</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>evaluation</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
@@ -508,6 +513,11 @@
       <c r="I2" t="n">
         <v>0.7900839664134346</v>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Ambiguous DR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -547,6 +557,11 @@
       <c r="I3" t="n">
         <v>0.998000799680128</v>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Ambiguous DR</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
@@ -586,6 +601,11 @@
       <c r="I4" t="n">
         <v>0.1261495401839264</v>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Confirmed DR</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
@@ -625,6 +645,11 @@
       <c r="I5" t="n">
         <v>0.9998000799680128</v>
       </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Ambiguous DR</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -664,6 +689,11 @@
       <c r="I6" t="n">
         <v>0.998000799680128</v>
       </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Ambiguous DR</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
@@ -703,6 +733,11 @@
       <c r="I7" t="n">
         <v>0.9632147141143542</v>
       </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Ambiguous DR</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
@@ -742,6 +777,11 @@
       <c r="I8" t="n">
         <v>0.9998000799680128</v>
       </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Ambiguous DR</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
@@ -781,6 +821,11 @@
       <c r="I9" t="n">
         <v>0.9998000799680128</v>
       </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Confirmed DR</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
@@ -820,6 +865,11 @@
       <c r="I10" t="n">
         <v>0.9998000799680128</v>
       </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Ambiguous DR</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -858,6 +908,11 @@
       </c>
       <c r="I11" t="n">
         <v>0.9998000799680128</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Ambiguous DR</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
writing update and thresholding rerun
</commit_message>
<xml_diff>
--- a/0_Threshold_OUTPUT/direct_A0A072Z841_Corynebacterium_glutamicum_ATCC_13032.xlsx
+++ b/0_Threshold_OUTPUT/direct_A0A072Z841_Corynebacterium_glutamicum_ATCC_13032.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,6 +474,11 @@
           <t>evaluation</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>correctness_%</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
@@ -518,6 +523,9 @@
           <t>Ambiguous DR</t>
         </is>
       </c>
+      <c r="K2" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -562,6 +570,9 @@
           <t>Ambiguous DR</t>
         </is>
       </c>
+      <c r="K3" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
@@ -606,6 +617,9 @@
           <t>Confirmed DR</t>
         </is>
       </c>
+      <c r="K4" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
@@ -650,6 +664,9 @@
           <t>Ambiguous DR</t>
         </is>
       </c>
+      <c r="K5" t="n">
+        <v>33.33</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -694,6 +711,9 @@
           <t>Ambiguous DR</t>
         </is>
       </c>
+      <c r="K6" t="n">
+        <v>33.33</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
@@ -738,6 +758,9 @@
           <t>Ambiguous DR</t>
         </is>
       </c>
+      <c r="K7" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
@@ -782,6 +805,9 @@
           <t>Ambiguous DR</t>
         </is>
       </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
@@ -826,6 +852,9 @@
           <t>Confirmed DR</t>
         </is>
       </c>
+      <c r="K9" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
@@ -870,6 +899,9 @@
           <t>Ambiguous DR</t>
         </is>
       </c>
+      <c r="K10" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -913,6 +945,9 @@
         <is>
           <t>Ambiguous DR</t>
         </is>
+      </c>
+      <c r="K11" t="n">
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>